<commit_message>
Adopt whole-number moderated grades with exact cohort mean 65
</commit_message>
<xml_diff>
--- a/RDM/RDM_Aug_26_Case_Study/RDM_Subcriterion_Percentage_Grades.xlsx
+++ b/RDM/RDM_Aug_26_Case_Study/RDM_Subcriterion_Percentage_Grades.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R827bde3363de4f16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subcriterion marks" sheetId="2" r:id="R495517313c054231"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distributions" sheetId="3" r:id="R97c6fce6b702473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mark audit" sheetId="4" r:id="R817441da7ed24bd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf91781a2913f455c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subcriterion marks" sheetId="2" r:id="Rebb10c42be84454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distributions" sheetId="3" r:id="R1eee7445c0fb4104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mark audit" sheetId="4" r:id="Re0089bfdc87d43e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,14 +16,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
     <x:numFmt numFmtId="202" formatCode="0"/>
     <x:numFmt numFmtId="203" formatCode="0.00%"/>
     <x:numFmt numFmtId="204" formatCode="0.0"/>
+    <x:numFmt numFmtId="205" formatCode="0.000000"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -50,13 +51,28 @@
       <x:color rgb="FF245EA6"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF234B62"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F5F7"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -75,7 +91,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="37">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -153,6 +169,18 @@
     <x:xf numFmtId="202" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="205" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -395,7 +423,7 @@
     </x:row>
     <x:row r="3" ht="38" customHeight="1">
       <x:c r="A3" s="4" t="str">
-        <x:v>17 submissions. Assessed marks use independent subcriterion judgements. The standardised comparison is a separate overall transformation.</x:v>
+        <x:v>17 submissions. Independent assessment is followed by overall standardisation and mean-preserving integer rounding. Moderated overall is the adjusted grade.</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -440,639 +468,639 @@
         <x:v>Assessed overall</x:v>
       </x:c>
       <x:c r="H5" s="7" t="str">
-        <x:v>Standardised comparison</x:v>
+        <x:v>Standardised before final rounding</x:v>
       </x:c>
       <x:c r="I5" s="7" t="str">
-        <x:v>Adjustment</x:v>
+        <x:v>Moderated overall</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="2" t="str">
         <x:v>Participant_555059_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B6" s="9" t="n">
+      <x:c r="B6" s="25" t="n">
         <x:f>'Subcriterion marks'!AE6</x:f>
         <x:v>59</x:v>
       </x:c>
-      <x:c r="C6" s="9" t="n">
+      <x:c r="C6" s="25" t="n">
         <x:f>'Subcriterion marks'!AF6</x:f>
         <x:v>73.33333333333333</x:v>
       </x:c>
-      <x:c r="D6" s="9" t="n">
+      <x:c r="D6" s="25" t="n">
         <x:f>'Subcriterion marks'!AG6</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="E6" s="9" t="n">
+      <x:c r="E6" s="25" t="n">
         <x:f>'Subcriterion marks'!AH6</x:f>
         <x:v>72.85714285714286</x:v>
       </x:c>
-      <x:c r="F6" s="9" t="n">
+      <x:c r="F6" s="25" t="n">
         <x:f>'Subcriterion marks'!AI6</x:f>
         <x:v>71.66666666666667</x:v>
       </x:c>
-      <x:c r="G6" s="9" t="n">
+      <x:c r="G6" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ6</x:f>
         <x:v>69.36904761904762</x:v>
       </x:c>
-      <x:c r="H6" s="9" t="n">
+      <x:c r="H6" s="25" t="n">
         <x:f>'Subcriterion marks'!AK6</x:f>
         <x:v>75.16853969752285</x:v>
       </x:c>
-      <x:c r="I6" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL6</x:f>
-        <x:v>5.799492078475225</x:v>
+      <x:c r="I6" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ6</x:f>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="8" t="str">
         <x:v>Participant_555060_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B7" s="10" t="n">
+      <x:c r="B7" s="26" t="n">
         <x:f>'Subcriterion marks'!AE7</x:f>
         <x:v>34</x:v>
       </x:c>
-      <x:c r="C7" s="10" t="n">
+      <x:c r="C7" s="26" t="n">
         <x:f>'Subcriterion marks'!AF7</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="D7" s="10" t="n">
+      <x:c r="D7" s="26" t="n">
         <x:f>'Subcriterion marks'!AG7</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E7" s="10" t="n">
+      <x:c r="E7" s="26" t="n">
         <x:f>'Subcriterion marks'!AH7</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="F7" s="10" t="n">
+      <x:c r="F7" s="26" t="n">
         <x:f>'Subcriterion marks'!AI7</x:f>
         <x:v>50.833333333333336</x:v>
       </x:c>
-      <x:c r="G7" s="10" t="n">
+      <x:c r="G7" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ7</x:f>
         <x:v>53.05357142857143</x:v>
       </x:c>
-      <x:c r="H7" s="10" t="n">
+      <x:c r="H7" s="26" t="n">
         <x:f>'Subcriterion marks'!AK7</x:f>
         <x:v>56.53534750414238</x:v>
       </x:c>
-      <x:c r="I7" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL7</x:f>
-        <x:v>3.4817760755709486</x:v>
+      <x:c r="I7" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ7</x:f>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="2" t="str">
         <x:v>Participant_555062_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B8" s="9" t="n">
+      <x:c r="B8" s="25" t="n">
         <x:f>'Subcriterion marks'!AE8</x:f>
         <x:v>57</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="n">
+      <x:c r="C8" s="25" t="n">
         <x:f>'Subcriterion marks'!AF8</x:f>
         <x:v>68.33333333333333</x:v>
       </x:c>
-      <x:c r="D8" s="9" t="n">
+      <x:c r="D8" s="25" t="n">
         <x:f>'Subcriterion marks'!AG8</x:f>
         <x:v>68</x:v>
       </x:c>
-      <x:c r="E8" s="9" t="n">
+      <x:c r="E8" s="25" t="n">
         <x:f>'Subcriterion marks'!AH8</x:f>
         <x:v>65.71428571428571</x:v>
       </x:c>
-      <x:c r="F8" s="9" t="n">
+      <x:c r="F8" s="25" t="n">
         <x:f>'Subcriterion marks'!AI8</x:f>
         <x:v>70.83333333333333</x:v>
       </x:c>
-      <x:c r="G8" s="9" t="n">
+      <x:c r="G8" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ8</x:f>
         <x:v>65.5297619047619</x:v>
       </x:c>
-      <x:c r="H8" s="9" t="n">
+      <x:c r="H8" s="25" t="n">
         <x:f>'Subcriterion marks'!AK8</x:f>
         <x:v>70.78385930178027</x:v>
       </x:c>
-      <x:c r="I8" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL8</x:f>
-        <x:v>5.25409739701837</x:v>
+      <x:c r="I8" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ8</x:f>
+        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="8" t="str">
         <x:v>Participant_555064_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B9" s="10" t="n">
+      <x:c r="B9" s="26" t="n">
         <x:f>'Subcriterion marks'!AE9</x:f>
         <x:v>62</x:v>
       </x:c>
-      <x:c r="C9" s="10" t="n">
+      <x:c r="C9" s="26" t="n">
         <x:f>'Subcriterion marks'!AF9</x:f>
         <x:v>80</x:v>
       </x:c>
-      <x:c r="D9" s="10" t="n">
+      <x:c r="D9" s="26" t="n">
         <x:f>'Subcriterion marks'!AG9</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="E9" s="10" t="n">
+      <x:c r="E9" s="26" t="n">
         <x:f>'Subcriterion marks'!AH9</x:f>
         <x:v>76.42857142857143</x:v>
       </x:c>
-      <x:c r="F9" s="10" t="n">
+      <x:c r="F9" s="26" t="n">
         <x:f>'Subcriterion marks'!AI9</x:f>
         <x:v>66.66666666666667</x:v>
       </x:c>
-      <x:c r="G9" s="10" t="n">
+      <x:c r="G9" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ9</x:f>
         <x:v>71.39285714285714</x:v>
       </x:c>
-      <x:c r="H9" s="10" t="n">
+      <x:c r="H9" s="26" t="n">
         <x:f>'Subcriterion marks'!AK9</x:f>
         <x:v>77.47984409217784</x:v>
       </x:c>
-      <x:c r="I9" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL9</x:f>
-        <x:v>6.086986949320703</x:v>
+      <x:c r="I9" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ9</x:f>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="2" t="str">
         <x:v>Participant_555065_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B10" s="9" t="n">
+      <x:c r="B10" s="25" t="n">
         <x:f>'Subcriterion marks'!AE10</x:f>
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C10" s="9" t="n">
+      <x:c r="C10" s="25" t="n">
         <x:f>'Subcriterion marks'!AF10</x:f>
         <x:v>69.16666666666667</x:v>
       </x:c>
-      <x:c r="D10" s="9" t="n">
+      <x:c r="D10" s="25" t="n">
         <x:f>'Subcriterion marks'!AG10</x:f>
         <x:v>68</x:v>
       </x:c>
-      <x:c r="E10" s="9" t="n">
+      <x:c r="E10" s="25" t="n">
         <x:f>'Subcriterion marks'!AH10</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="F10" s="9" t="n">
+      <x:c r="F10" s="25" t="n">
         <x:f>'Subcriterion marks'!AI10</x:f>
         <x:v>67.5</x:v>
       </x:c>
-      <x:c r="G10" s="9" t="n">
+      <x:c r="G10" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ10</x:f>
         <x:v>68.5952380952381</x:v>
       </x:c>
-      <x:c r="H10" s="9" t="n">
+      <x:c r="H10" s="25" t="n">
         <x:f>'Subcriterion marks'!AK10</x:f>
         <x:v>74.28480566427241</x:v>
       </x:c>
-      <x:c r="I10" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL10</x:f>
-        <x:v>5.68956756903431</x:v>
+      <x:c r="I10" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ10</x:f>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="8" t="str">
         <x:v>Participant_555066_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B11" s="10" t="n">
+      <x:c r="B11" s="26" t="n">
         <x:f>'Subcriterion marks'!AE11</x:f>
         <x:v>59</x:v>
       </x:c>
-      <x:c r="C11" s="10" t="n">
+      <x:c r="C11" s="26" t="n">
         <x:f>'Subcriterion marks'!AF11</x:f>
         <x:v>74.16666666666667</x:v>
       </x:c>
-      <x:c r="D11" s="10" t="n">
+      <x:c r="D11" s="26" t="n">
         <x:f>'Subcriterion marks'!AG11</x:f>
         <x:v>74</x:v>
       </x:c>
-      <x:c r="E11" s="10" t="n">
+      <x:c r="E11" s="26" t="n">
         <x:f>'Subcriterion marks'!AH11</x:f>
         <x:v>70.71428571428571</x:v>
       </x:c>
-      <x:c r="F11" s="10" t="n">
+      <x:c r="F11" s="26" t="n">
         <x:f>'Subcriterion marks'!AI11</x:f>
         <x:v>68.33333333333333</x:v>
       </x:c>
-      <x:c r="G11" s="10" t="n">
+      <x:c r="G11" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ11</x:f>
         <x:v>69.11309523809524</x:v>
       </x:c>
-      <x:c r="H11" s="10" t="n">
+      <x:c r="H11" s="26" t="n">
         <x:f>'Subcriterion marks'!AK11</x:f>
         <x:v>74.87622767114001</x:v>
       </x:c>
-      <x:c r="I11" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL11</x:f>
-        <x:v>5.763132433044774</x:v>
+      <x:c r="I11" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ11</x:f>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="2" t="str">
         <x:v>Participant_555069_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B12" s="9" t="n">
+      <x:c r="B12" s="25" t="n">
         <x:f>'Subcriterion marks'!AE12</x:f>
         <x:v>43</x:v>
       </x:c>
-      <x:c r="C12" s="9" t="n">
+      <x:c r="C12" s="25" t="n">
         <x:f>'Subcriterion marks'!AF12</x:f>
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D12" s="9" t="n">
+      <x:c r="D12" s="25" t="n">
         <x:f>'Subcriterion marks'!AG12</x:f>
         <x:v>49</x:v>
       </x:c>
-      <x:c r="E12" s="9" t="n">
+      <x:c r="E12" s="25" t="n">
         <x:f>'Subcriterion marks'!AH12</x:f>
         <x:v>57.857142857142854</x:v>
       </x:c>
-      <x:c r="F12" s="9" t="n">
+      <x:c r="F12" s="25" t="n">
         <x:f>'Subcriterion marks'!AI12</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G12" s="9" t="n">
+      <x:c r="G12" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ12</x:f>
         <x:v>49.035714285714285</x:v>
       </x:c>
-      <x:c r="H12" s="9" t="n">
+      <x:c r="H12" s="25" t="n">
         <x:f>'Subcriterion marks'!AK12</x:f>
         <x:v>51.94672848534201</x:v>
       </x:c>
-      <x:c r="I12" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL12</x:f>
-        <x:v>2.911014199627722</x:v>
+      <x:c r="I12" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ12</x:f>
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="8" t="str">
         <x:v>Participant_555070_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B13" s="10" t="n">
+      <x:c r="B13" s="26" t="n">
         <x:f>'Subcriterion marks'!AE13</x:f>
         <x:v>44</x:v>
       </x:c>
-      <x:c r="C13" s="10" t="n">
+      <x:c r="C13" s="26" t="n">
         <x:f>'Subcriterion marks'!AF13</x:f>
         <x:v>48.333333333333336</x:v>
       </x:c>
-      <x:c r="D13" s="10" t="n">
+      <x:c r="D13" s="26" t="n">
         <x:f>'Subcriterion marks'!AG13</x:f>
         <x:v>52</x:v>
       </x:c>
-      <x:c r="E13" s="10" t="n">
+      <x:c r="E13" s="26" t="n">
         <x:f>'Subcriterion marks'!AH13</x:f>
         <x:v>60.714285714285715</x:v>
       </x:c>
-      <x:c r="F13" s="10" t="n">
+      <x:c r="F13" s="26" t="n">
         <x:f>'Subcriterion marks'!AI13</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="G13" s="10" t="n">
+      <x:c r="G13" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ13</x:f>
         <x:v>46.654761904761905</x:v>
       </x:c>
-      <x:c r="H13" s="10" t="n">
+      <x:c r="H13" s="26" t="n">
         <x:f>'Subcriterion marks'!AK13</x:f>
         <x:v>49.22754684457142</x:v>
       </x:c>
-      <x:c r="I13" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL13</x:f>
-        <x:v>2.572784939809516</x:v>
+      <x:c r="I13" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ13</x:f>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="2" t="str">
         <x:v>Participant_555071_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B14" s="9" t="n">
+      <x:c r="B14" s="25" t="n">
         <x:f>'Subcriterion marks'!AE14</x:f>
         <x:v>43</x:v>
       </x:c>
-      <x:c r="C14" s="9" t="n">
+      <x:c r="C14" s="25" t="n">
         <x:f>'Subcriterion marks'!AF14</x:f>
         <x:v>54.166666666666664</x:v>
       </x:c>
-      <x:c r="D14" s="9" t="n">
+      <x:c r="D14" s="25" t="n">
         <x:f>'Subcriterion marks'!AG14</x:f>
         <x:v>53</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="n">
+      <x:c r="E14" s="25" t="n">
         <x:f>'Subcriterion marks'!AH14</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="F14" s="9" t="n">
+      <x:c r="F14" s="25" t="n">
         <x:f>'Subcriterion marks'!AI14</x:f>
         <x:v>59.166666666666664</x:v>
       </x:c>
-      <x:c r="G14" s="9" t="n">
+      <x:c r="G14" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ14</x:f>
         <x:v>52.416666666666664</x:v>
       </x:c>
-      <x:c r="H14" s="9" t="n">
+      <x:c r="H14" s="25" t="n">
         <x:f>'Subcriterion marks'!AK14</x:f>
         <x:v>55.807966415236244</x:v>
       </x:c>
-      <x:c r="I14" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL14</x:f>
-        <x:v>3.3912997485695797</x:v>
+      <x:c r="I14" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ14</x:f>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="8" t="str">
         <x:v>Participant_555072_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B15" s="10" t="n">
+      <x:c r="B15" s="26" t="n">
         <x:f>'Subcriterion marks'!AE15</x:f>
         <x:v>72</x:v>
       </x:c>
-      <x:c r="C15" s="10" t="n">
+      <x:c r="C15" s="26" t="n">
         <x:f>'Subcriterion marks'!AF15</x:f>
         <x:v>82.5</x:v>
       </x:c>
-      <x:c r="D15" s="10" t="n">
+      <x:c r="D15" s="26" t="n">
         <x:f>'Subcriterion marks'!AG15</x:f>
         <x:v>74</x:v>
       </x:c>
-      <x:c r="E15" s="10" t="n">
+      <x:c r="E15" s="26" t="n">
         <x:f>'Subcriterion marks'!AH15</x:f>
         <x:v>76.42857142857143</x:v>
       </x:c>
-      <x:c r="F15" s="10" t="n">
+      <x:c r="F15" s="26" t="n">
         <x:f>'Subcriterion marks'!AI15</x:f>
         <x:v>71.66666666666667</x:v>
       </x:c>
-      <x:c r="G15" s="10" t="n">
+      <x:c r="G15" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ15</x:f>
         <x:v>75.51785714285714</x:v>
       </x:c>
-      <x:c r="H15" s="10" t="n">
+      <x:c r="H15" s="26" t="n">
         <x:f>'Subcriterion marks'!AK15</x:f>
         <x:v>82.19082628481289</x:v>
       </x:c>
-      <x:c r="I15" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL15</x:f>
-        <x:v>6.672969141955747</x:v>
+      <x:c r="I15" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ15</x:f>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="2" t="str">
         <x:v>Participant_555073_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B16" s="9" t="n">
+      <x:c r="B16" s="25" t="n">
         <x:f>'Subcriterion marks'!AE16</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C16" s="9" t="n">
+      <x:c r="C16" s="25" t="n">
         <x:f>'Subcriterion marks'!AF16</x:f>
         <x:v>75</x:v>
       </x:c>
-      <x:c r="D16" s="9" t="n">
+      <x:c r="D16" s="25" t="n">
         <x:f>'Subcriterion marks'!AG16</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="E16" s="9" t="n">
+      <x:c r="E16" s="25" t="n">
         <x:f>'Subcriterion marks'!AH16</x:f>
         <x:v>76.42857142857143</x:v>
       </x:c>
-      <x:c r="F16" s="9" t="n">
+      <x:c r="F16" s="25" t="n">
         <x:f>'Subcriterion marks'!AI16</x:f>
         <x:v>73.33333333333333</x:v>
       </x:c>
-      <x:c r="G16" s="9" t="n">
+      <x:c r="G16" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ16</x:f>
         <x:v>70.64285714285714</x:v>
       </x:c>
-      <x:c r="H16" s="9" t="n">
+      <x:c r="H16" s="25" t="n">
         <x:f>'Subcriterion marks'!AK16</x:f>
         <x:v>76.6233018753351</x:v>
       </x:c>
-      <x:c r="I16" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL16</x:f>
-        <x:v>5.980444732477963</x:v>
+      <x:c r="I16" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ16</x:f>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="8" t="str">
         <x:v>Participant_555074_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B17" s="10" t="n">
+      <x:c r="B17" s="26" t="n">
         <x:f>'Subcriterion marks'!AE17</x:f>
         <x:v>52</x:v>
       </x:c>
-      <x:c r="C17" s="10" t="n">
+      <x:c r="C17" s="26" t="n">
         <x:f>'Subcriterion marks'!AF17</x:f>
         <x:v>51.666666666666664</x:v>
       </x:c>
-      <x:c r="D17" s="10" t="n">
+      <x:c r="D17" s="26" t="n">
         <x:f>'Subcriterion marks'!AG17</x:f>
         <x:v>63</x:v>
       </x:c>
-      <x:c r="E17" s="10" t="n">
+      <x:c r="E17" s="26" t="n">
         <x:f>'Subcriterion marks'!AH17</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="F17" s="10" t="n">
+      <x:c r="F17" s="26" t="n">
         <x:f>'Subcriterion marks'!AI17</x:f>
         <x:v>60.833333333333336</x:v>
       </x:c>
-      <x:c r="G17" s="10" t="n">
+      <x:c r="G17" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ17</x:f>
         <x:v>57.720238095238095</x:v>
       </x:c>
-      <x:c r="H17" s="10" t="n">
+      <x:c r="H17" s="26" t="n">
         <x:f>'Subcriterion marks'!AK17</x:f>
         <x:v>61.864943520052734</x:v>
       </x:c>
-      <x:c r="I17" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL17</x:f>
-        <x:v>4.144705424814639</x:v>
+      <x:c r="I17" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ17</x:f>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="2" t="str">
         <x:v>Participant_555076_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B18" s="9" t="n">
+      <x:c r="B18" s="25" t="n">
         <x:f>'Subcriterion marks'!AE18</x:f>
         <x:v>37</x:v>
       </x:c>
-      <x:c r="C18" s="9" t="n">
+      <x:c r="C18" s="25" t="n">
         <x:f>'Subcriterion marks'!AF18</x:f>
         <x:v>55.833333333333336</x:v>
       </x:c>
-      <x:c r="D18" s="9" t="n">
+      <x:c r="D18" s="25" t="n">
         <x:f>'Subcriterion marks'!AG18</x:f>
         <x:v>57</x:v>
       </x:c>
-      <x:c r="E18" s="9" t="n">
+      <x:c r="E18" s="25" t="n">
         <x:f>'Subcriterion marks'!AH18</x:f>
         <x:v>57.857142857142854</x:v>
       </x:c>
-      <x:c r="F18" s="9" t="n">
+      <x:c r="F18" s="25" t="n">
         <x:f>'Subcriterion marks'!AI18</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="G18" s="9" t="n">
+      <x:c r="G18" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ18</x:f>
         <x:v>52.24404761904762</x:v>
       </x:c>
-      <x:c r="H18" s="9" t="n">
+      <x:c r="H18" s="25" t="n">
         <x:f>'Subcriterion marks'!AK18</x:f>
         <x:v>55.61082574628038</x:v>
       </x:c>
-      <x:c r="I18" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL18</x:f>
-        <x:v>3.366778127232763</x:v>
+      <x:c r="I18" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ18</x:f>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="8" t="str">
         <x:v>Participant_555077_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B19" s="10" t="n">
+      <x:c r="B19" s="26" t="n">
         <x:f>'Subcriterion marks'!AE19</x:f>
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C19" s="10" t="n">
+      <x:c r="C19" s="26" t="n">
         <x:f>'Subcriterion marks'!AF19</x:f>
         <x:v>62.5</x:v>
       </x:c>
-      <x:c r="D19" s="10" t="n">
+      <x:c r="D19" s="26" t="n">
         <x:f>'Subcriterion marks'!AG19</x:f>
         <x:v>63</x:v>
       </x:c>
-      <x:c r="E19" s="10" t="n">
+      <x:c r="E19" s="26" t="n">
         <x:f>'Subcriterion marks'!AH19</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="F19" s="10" t="n">
+      <x:c r="F19" s="26" t="n">
         <x:f>'Subcriterion marks'!AI19</x:f>
         <x:v>62.5</x:v>
       </x:c>
-      <x:c r="G19" s="10" t="n">
+      <x:c r="G19" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ19</x:f>
         <x:v>57.42857142857143</x:v>
       </x:c>
-      <x:c r="H19" s="10" t="n">
+      <x:c r="H19" s="26" t="n">
         <x:f>'Subcriterion marks'!AK19</x:f>
         <x:v>61.53184376905834</x:v>
       </x:c>
-      <x:c r="I19" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL19</x:f>
-        <x:v>4.10327234048691</x:v>
+      <x:c r="I19" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ19</x:f>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="2" t="str">
         <x:v>Participant_555078_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B20" s="9" t="n">
+      <x:c r="B20" s="25" t="n">
         <x:f>'Subcriterion marks'!AE20</x:f>
         <x:v>39</x:v>
       </x:c>
-      <x:c r="C20" s="9" t="n">
+      <x:c r="C20" s="25" t="n">
         <x:f>'Subcriterion marks'!AF20</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="D20" s="9" t="n">
+      <x:c r="D20" s="25" t="n">
         <x:f>'Subcriterion marks'!AG20</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E20" s="9" t="n">
+      <x:c r="E20" s="25" t="n">
         <x:f>'Subcriterion marks'!AH20</x:f>
         <x:v>57.857142857142854</x:v>
       </x:c>
-      <x:c r="F20" s="9" t="n">
+      <x:c r="F20" s="25" t="n">
         <x:f>'Subcriterion marks'!AI20</x:f>
         <x:v>61.666666666666664</x:v>
       </x:c>
-      <x:c r="G20" s="9" t="n">
+      <x:c r="G20" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ20</x:f>
         <x:v>54.785714285714285</x:v>
       </x:c>
-      <x:c r="H20" s="9" t="n">
+      <x:c r="H20" s="25" t="n">
         <x:f>'Subcriterion marks'!AK20</x:f>
         <x:v>58.51355214780298</x:v>
       </x:c>
-      <x:c r="I20" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL20</x:f>
-        <x:v>3.7278378620886983</x:v>
+      <x:c r="I20" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ20</x:f>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="8" t="str">
         <x:v>Participant_555079_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B21" s="10" t="n">
+      <x:c r="B21" s="26" t="n">
         <x:f>'Subcriterion marks'!AE21</x:f>
         <x:v>41</x:v>
       </x:c>
-      <x:c r="C21" s="10" t="n">
+      <x:c r="C21" s="26" t="n">
         <x:f>'Subcriterion marks'!AF21</x:f>
         <x:v>70</x:v>
       </x:c>
-      <x:c r="D21" s="10" t="n">
+      <x:c r="D21" s="26" t="n">
         <x:f>'Subcriterion marks'!AG21</x:f>
         <x:v>67</x:v>
       </x:c>
-      <x:c r="E21" s="10" t="n">
+      <x:c r="E21" s="26" t="n">
         <x:f>'Subcriterion marks'!AH21</x:f>
         <x:v>61.42857142857143</x:v>
       </x:c>
-      <x:c r="F21" s="10" t="n">
+      <x:c r="F21" s="26" t="n">
         <x:f>'Subcriterion marks'!AI21</x:f>
         <x:v>69.16666666666667</x:v>
       </x:c>
-      <x:c r="G21" s="10" t="n">
+      <x:c r="G21" s="26" t="n">
         <x:f>'Subcriterion marks'!AJ21</x:f>
         <x:v>61.017857142857146</x:v>
       </x:c>
-      <x:c r="H21" s="10" t="n">
+      <x:c r="H21" s="26" t="n">
         <x:f>'Subcriterion marks'!AK21</x:f>
         <x:v>65.63101009252</x:v>
       </x:c>
-      <x:c r="I21" s="10" t="n">
-        <x:f>'Subcriterion marks'!AL21</x:f>
-        <x:v>4.6131529496628545</x:v>
+      <x:c r="I21" s="26" t="n">
+        <x:f>'Subcriterion marks'!AQ21</x:f>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="2" t="str">
         <x:v>Participant_564388_assignsubmission_file</x:v>
       </x:c>
-      <x:c r="B22" s="9" t="n">
+      <x:c r="B22" s="25" t="n">
         <x:f>'Subcriterion marks'!AE22</x:f>
         <x:v>47</x:v>
       </x:c>
-      <x:c r="C22" s="9" t="n">
+      <x:c r="C22" s="25" t="n">
         <x:f>'Subcriterion marks'!AF22</x:f>
         <x:v>52.5</x:v>
       </x:c>
-      <x:c r="D22" s="9" t="n">
+      <x:c r="D22" s="25" t="n">
         <x:f>'Subcriterion marks'!AG22</x:f>
         <x:v>58</x:v>
       </x:c>
-      <x:c r="E22" s="9" t="n">
+      <x:c r="E22" s="25" t="n">
         <x:f>'Subcriterion marks'!AH22</x:f>
         <x:v>61.42857142857143</x:v>
       </x:c>
-      <x:c r="F22" s="9" t="n">
+      <x:c r="F22" s="25" t="n">
         <x:f>'Subcriterion marks'!AI22</x:f>
         <x:v>52.5</x:v>
       </x:c>
-      <x:c r="G22" s="9" t="n">
+      <x:c r="G22" s="25" t="n">
         <x:f>'Subcriterion marks'!AJ22</x:f>
         <x:v>53.392857142857146</x:v>
       </x:c>
-      <x:c r="H22" s="9" t="n">
+      <x:c r="H22" s="25" t="n">
         <x:f>'Subcriterion marks'!AK22</x:f>
         <x:v>56.92283088795219</x:v>
       </x:c>
-      <x:c r="I22" s="9" t="n">
-        <x:f>'Subcriterion marks'!AL22</x:f>
-        <x:v>3.5299737450950417</x:v>
+      <x:c r="I22" s="25" t="n">
+        <x:f>'Subcriterion marks'!AQ22</x:f>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
@@ -1133,7 +1161,7 @@
       </x:c>
       <x:c r="I25" s="9" t="n">
         <x:f>AVERAGE(I6:I22)</x:f>
-        <x:v>4.534663865546222</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
@@ -1170,7 +1198,7 @@
       </x:c>
       <x:c r="I26" s="9" t="n">
         <x:f>STDEV.P(I6:I22)</x:f>
-        <x:v>1.2438641639341088</x:v>
+        <x:v>9.952829925674997</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
@@ -1207,7 +1235,7 @@
       </x:c>
       <x:c r="I27" s="9" t="n">
         <x:f>MIN(I6:I22)</x:f>
-        <x:v>2.572784939809516</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
@@ -1244,7 +1272,7 @@
       </x:c>
       <x:c r="I28" s="9" t="n">
         <x:f>MAX(I6:I22)</x:f>
-        <x:v>6.672969141955747</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
@@ -1362,7 +1390,7 @@
     </x:row>
     <x:row r="36" ht="46" customHeight="1">
       <x:c r="A36" s="7" t="str">
-        <x:v>Standardisation comparison</x:v>
+        <x:v>Overall moderation target</x:v>
       </x:c>
       <x:c r="B36" s="7" t="str">
         <x:v>Target</x:v>
@@ -1442,7 +1470,7 @@
     </x:row>
     <x:row r="42" ht="40" customHeight="1">
       <x:c r="A42" s="4" t="str">
-        <x:v>Standardised comparison = target mean + target SD × (assessed overall − cohort mean) / population SD. It does not change subcriterion marks or impose a normal distribution.</x:v>
+        <x:v>Overall standardisation = 65 + 10 × (assessed overall − cohort mean) / population SD. The moderated overall applies mean-preserving integer rounding to this result.</x:v>
       </x:c>
       <x:c r="B42" s="4"/>
       <x:c r="C42" s="4"/>
@@ -1455,7 +1483,7 @@
     </x:row>
     <x:row r="43" ht="40" customHeight="1">
       <x:c r="A43" s="4" t="str">
-        <x:v>Marks are provisional for inspection. The comparison does not equal the weighted sum of unchanged subcriterion marks. No additional caps or penalties are applied.</x:v>
+        <x:v>Moderated overall is the adjusted grade for inspection. It does not equal the weighted sum of unchanged subcriterion marks. No additional caps or penalties are applied.</x:v>
       </x:c>
       <x:c r="B43" s="4"/>
       <x:c r="C43" s="4"/>
@@ -1611,7 +1639,7 @@
     </x:row>
     <x:row r="55" ht="40" customHeight="1">
       <x:c r="A55" s="4" t="str">
-        <x:v>All marks are stored on a 0–100 scale. Displayed totals use two decimals; calculations retain full precision. Changes to marks or weights recalculate the assessment and comparison.</x:v>
+        <x:v>All displayed student marks are whole numbers. Criterion averages and standardisation retain full precision internally; final moderated grades are actual integers, not just formatted decimals.</x:v>
       </x:c>
       <x:c r="B55" s="4"/>
       <x:c r="C55" s="4"/>
@@ -1624,7 +1652,7 @@
     </x:row>
     <x:row r="56" ht="40" customHeight="1">
       <x:c r="A56" s="4" t="str">
-        <x:v>Full reusable method: RDM/RDM_Aug_26_Case_Study/GRADING_METHOD_Independent_Subcriteria.md in HRP-Transfer-Lab/uoe-feedback.</x:v>
+        <x:v>Method v1.1: GRADING_METHOD_Independent_Subcriteria.md. Round down each standardised score, then round up the largest fractional remainders until the total equals 65 × N.</x:v>
       </x:c>
       <x:c r="B56" s="4"/>
       <x:c r="C56" s="4"/>
@@ -1635,38 +1663,44 @@
       <x:c r="H56" s="4"/>
       <x:c r="I56" s="4"/>
     </x:row>
-    <x:row r="57" ht="25" customHeight="1">
-      <x:c r="A57" s="2"/>
-      <x:c r="B57" s="2"/>
-      <x:c r="C57" s="2"/>
-      <x:c r="D57" s="2"/>
-      <x:c r="E57" s="2"/>
-      <x:c r="F57" s="2"/>
-      <x:c r="G57" s="2"/>
-      <x:c r="H57" s="2"/>
-      <x:c r="I57" s="2"/>
-    </x:row>
-    <x:row r="58" ht="25" customHeight="1">
-      <x:c r="A58" s="2"/>
-      <x:c r="B58" s="2"/>
-      <x:c r="C58" s="2"/>
-      <x:c r="D58" s="2"/>
-      <x:c r="E58" s="2"/>
-      <x:c r="F58" s="2"/>
-      <x:c r="G58" s="2"/>
-      <x:c r="H58" s="2"/>
-      <x:c r="I58" s="2"/>
-    </x:row>
-    <x:row r="59" ht="25" customHeight="1">
-      <x:c r="A59" s="2"/>
-      <x:c r="B59" s="2"/>
-      <x:c r="C59" s="2"/>
-      <x:c r="D59" s="2"/>
-      <x:c r="E59" s="2"/>
-      <x:c r="F59" s="2"/>
-      <x:c r="G59" s="2"/>
-      <x:c r="H59" s="2"/>
-      <x:c r="I59" s="2"/>
+    <x:row r="57" ht="40" customHeight="1">
+      <x:c r="A57" s="4" t="str">
+        <x:v>For 17 students the required total is 1,105. Ordinary nearest-integer rounding gives 1,107, so two borderline scores round down to preserve the exact mean of 65.</x:v>
+      </x:c>
+      <x:c r="B57" s="4"/>
+      <x:c r="C57" s="4"/>
+      <x:c r="D57" s="4"/>
+      <x:c r="E57" s="4"/>
+      <x:c r="F57" s="4"/>
+      <x:c r="G57" s="4"/>
+      <x:c r="H57" s="4"/>
+      <x:c r="I57" s="4"/>
+    </x:row>
+    <x:row r="58" ht="40" customHeight="1">
+      <x:c r="A58" s="4" t="str">
+        <x:v>Integer rounding changes the SD slightly from 10. Statistics retain decimals for transparency. Subcriterion marks and preserved Stage 1 codes are unchanged.</x:v>
+      </x:c>
+      <x:c r="B58" s="4"/>
+      <x:c r="C58" s="4"/>
+      <x:c r="D58" s="4"/>
+      <x:c r="E58" s="4"/>
+      <x:c r="F58" s="4"/>
+      <x:c r="G58" s="4"/>
+      <x:c r="H58" s="4"/>
+      <x:c r="I58" s="4"/>
+    </x:row>
+    <x:row r="59" ht="40" customHeight="1">
+      <x:c r="A59" s="4" t="str">
+        <x:v>Remainder ties use the existing ascending participant-ID order. Identical underlying scores that would be split by rounding require manual review; none occur in this cohort.</x:v>
+      </x:c>
+      <x:c r="B59" s="4"/>
+      <x:c r="C59" s="4"/>
+      <x:c r="D59" s="4"/>
+      <x:c r="E59" s="4"/>
+      <x:c r="F59" s="4"/>
+      <x:c r="G59" s="4"/>
+      <x:c r="H59" s="4"/>
+      <x:c r="I59" s="4"/>
     </x:row>
     <x:row r="60" ht="25" customHeight="1">
       <x:c r="A60" s="2"/>
@@ -1731,6 +1765,9 @@
     <x:mergeCell ref="A54:I54"/>
     <x:mergeCell ref="A55:I55"/>
     <x:mergeCell ref="A56:I56"/>
+    <x:mergeCell ref="A57:I57"/>
+    <x:mergeCell ref="A58:I58"/>
+    <x:mergeCell ref="A59:I59"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1785,6 +1822,10 @@
     <x:col min="40" max="40" width="3" hidden="0" customWidth="1"/>
     <x:col min="41" max="41" width="90" hidden="0" customWidth="1"/>
     <x:col min="42" max="42" width="45" hidden="0" customWidth="1"/>
+    <x:col min="43" max="43" width="19" hidden="0" customWidth="1"/>
+    <x:col min="44" max="44" width="19" hidden="0" customWidth="1"/>
+    <x:col min="45" max="45" width="19" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="19" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
@@ -2092,6 +2133,18 @@
       <x:c r="AP5" s="7" t="str">
         <x:v>Source blob SHA</x:v>
       </x:c>
+      <x:c r="AQ5" s="30" t="str">
+        <x:v>Moderated overall</x:v>
+      </x:c>
+      <x:c r="AR5" s="30" t="str">
+        <x:v>Rounding floor</x:v>
+      </x:c>
+      <x:c r="AS5" s="30" t="str">
+        <x:v>Fractional remainder</x:v>
+      </x:c>
+      <x:c r="AT5" s="30" t="str">
+        <x:v>Remainder priority</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="2" t="str">
@@ -2184,35 +2237,35 @@
       <x:c r="AD6" s="18" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="AE6" s="9" t="n">
+      <x:c r="AE6" s="25" t="n">
         <x:f>AVERAGE(B6:F6)</x:f>
         <x:v>59</x:v>
       </x:c>
-      <x:c r="AF6" s="9" t="n">
+      <x:c r="AF6" s="25" t="n">
         <x:f>AVERAGE(G6:L6)</x:f>
         <x:v>73.33333333333333</x:v>
       </x:c>
-      <x:c r="AG6" s="9" t="n">
+      <x:c r="AG6" s="25" t="n">
         <x:f>AVERAGE(M6:Q6)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="AH6" s="9" t="n">
+      <x:c r="AH6" s="25" t="n">
         <x:f>AVERAGE(R6:X6)</x:f>
         <x:v>72.85714285714286</x:v>
       </x:c>
-      <x:c r="AI6" s="9" t="n">
+      <x:c r="AI6" s="25" t="n">
         <x:f>AVERAGE(Y6:AD6)</x:f>
         <x:v>71.66666666666667</x:v>
       </x:c>
-      <x:c r="AJ6" s="9" t="n">
+      <x:c r="AJ6" s="25" t="n">
         <x:f>SUMPRODUCT(AE6:AI6,Overview!$B$34:$F$34)</x:f>
         <x:v>69.36904761904762</x:v>
       </x:c>
-      <x:c r="AK6" s="9" t="n">
+      <x:c r="AK6" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ6-$AJ$25)/$AJ$26)</x:f>
         <x:v>75.16853969752285</x:v>
       </x:c>
-      <x:c r="AL6" s="9" t="n">
+      <x:c r="AL6" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK6-AJ6)</x:f>
         <x:v>5.799492078475225</x:v>
       </x:c>
@@ -2227,6 +2280,22 @@
       <x:c r="AP6" s="2" t="str">
         <x:v>fd1b5a5153ec162fae5bd4e1a5a8c13d15275401</x:v>
       </x:c>
+      <x:c r="AQ6" s="32" t="n">
+        <x:f>AR6+IF(AT6&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="AR6" s="32" t="n">
+        <x:f>INT(AK6)</x:f>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="AS6" s="34" t="n">
+        <x:f>AK6-AR6</x:f>
+        <x:v>0.1685396975228457</x:v>
+      </x:c>
+      <x:c r="AT6" s="32" t="n">
+        <x:f>RANK(AS6,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS6,AS6)-1</x:f>
+        <x:v>17</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="8" t="str">
@@ -2319,35 +2388,35 @@
       <x:c r="AD7" s="19" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="AE7" s="10" t="n">
+      <x:c r="AE7" s="26" t="n">
         <x:f>AVERAGE(B7:F7)</x:f>
         <x:v>34</x:v>
       </x:c>
-      <x:c r="AF7" s="10" t="n">
+      <x:c r="AF7" s="26" t="n">
         <x:f>AVERAGE(G7:L7)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AG7" s="10" t="n">
+      <x:c r="AG7" s="26" t="n">
         <x:f>AVERAGE(M7:Q7)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AH7" s="10" t="n">
+      <x:c r="AH7" s="26" t="n">
         <x:f>AVERAGE(R7:X7)</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="AI7" s="10" t="n">
+      <x:c r="AI7" s="26" t="n">
         <x:f>AVERAGE(Y7:AD7)</x:f>
         <x:v>50.833333333333336</x:v>
       </x:c>
-      <x:c r="AJ7" s="10" t="n">
+      <x:c r="AJ7" s="26" t="n">
         <x:f>SUMPRODUCT(AE7:AI7,Overview!$B$34:$F$34)</x:f>
         <x:v>53.05357142857143</x:v>
       </x:c>
-      <x:c r="AK7" s="10" t="n">
+      <x:c r="AK7" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ7-$AJ$25)/$AJ$26)</x:f>
         <x:v>56.53534750414238</x:v>
       </x:c>
-      <x:c r="AL7" s="10" t="n">
+      <x:c r="AL7" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK7-AJ7)</x:f>
         <x:v>3.4817760755709486</x:v>
       </x:c>
@@ -2362,6 +2431,22 @@
       <x:c r="AP7" s="8" t="str">
         <x:v>35e833fec71aedef1c7def2908626bf4f4e1c8e4</x:v>
       </x:c>
+      <x:c r="AQ7" s="33" t="n">
+        <x:f>AR7+IF(AT7&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="AR7" s="33" t="n">
+        <x:f>INT(AK7)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="AS7" s="35" t="n">
+        <x:f>AK7-AR7</x:f>
+        <x:v>0.5353475041423792</x:v>
+      </x:c>
+      <x:c r="AT7" s="33" t="n">
+        <x:f>RANK(AS7,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS7,AS7)-1</x:f>
+        <x:v>10</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="2" t="str">
@@ -2454,35 +2539,35 @@
       <x:c r="AD8" s="18" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="AE8" s="9" t="n">
+      <x:c r="AE8" s="25" t="n">
         <x:f>AVERAGE(B8:F8)</x:f>
         <x:v>57</x:v>
       </x:c>
-      <x:c r="AF8" s="9" t="n">
+      <x:c r="AF8" s="25" t="n">
         <x:f>AVERAGE(G8:L8)</x:f>
         <x:v>68.33333333333333</x:v>
       </x:c>
-      <x:c r="AG8" s="9" t="n">
+      <x:c r="AG8" s="25" t="n">
         <x:f>AVERAGE(M8:Q8)</x:f>
         <x:v>68</x:v>
       </x:c>
-      <x:c r="AH8" s="9" t="n">
+      <x:c r="AH8" s="25" t="n">
         <x:f>AVERAGE(R8:X8)</x:f>
         <x:v>65.71428571428571</x:v>
       </x:c>
-      <x:c r="AI8" s="9" t="n">
+      <x:c r="AI8" s="25" t="n">
         <x:f>AVERAGE(Y8:AD8)</x:f>
         <x:v>70.83333333333333</x:v>
       </x:c>
-      <x:c r="AJ8" s="9" t="n">
+      <x:c r="AJ8" s="25" t="n">
         <x:f>SUMPRODUCT(AE8:AI8,Overview!$B$34:$F$34)</x:f>
         <x:v>65.5297619047619</x:v>
       </x:c>
-      <x:c r="AK8" s="9" t="n">
+      <x:c r="AK8" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ8-$AJ$25)/$AJ$26)</x:f>
         <x:v>70.78385930178027</x:v>
       </x:c>
-      <x:c r="AL8" s="9" t="n">
+      <x:c r="AL8" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK8-AJ8)</x:f>
         <x:v>5.25409739701837</x:v>
       </x:c>
@@ -2497,6 +2582,22 @@
       <x:c r="AP8" s="2" t="str">
         <x:v>8b668c9c330a5ad5f5fccb8ec36c0ed190024f12</x:v>
       </x:c>
+      <x:c r="AQ8" s="32" t="n">
+        <x:f>AR8+IF(AT8&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="AR8" s="32" t="n">
+        <x:f>INT(AK8)</x:f>
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="AS8" s="34" t="n">
+        <x:f>AK8-AR8</x:f>
+        <x:v>0.783859301780268</x:v>
+      </x:c>
+      <x:c r="AT8" s="32" t="n">
+        <x:f>RANK(AS8,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS8,AS8)-1</x:f>
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="8" t="str">
@@ -2589,35 +2690,35 @@
       <x:c r="AD9" s="19" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="AE9" s="10" t="n">
+      <x:c r="AE9" s="26" t="n">
         <x:f>AVERAGE(B9:F9)</x:f>
         <x:v>62</x:v>
       </x:c>
-      <x:c r="AF9" s="10" t="n">
+      <x:c r="AF9" s="26" t="n">
         <x:f>AVERAGE(G9:L9)</x:f>
         <x:v>80</x:v>
       </x:c>
-      <x:c r="AG9" s="10" t="n">
+      <x:c r="AG9" s="26" t="n">
         <x:f>AVERAGE(M9:Q9)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="AH9" s="10" t="n">
+      <x:c r="AH9" s="26" t="n">
         <x:f>AVERAGE(R9:X9)</x:f>
         <x:v>76.42857142857143</x:v>
       </x:c>
-      <x:c r="AI9" s="10" t="n">
+      <x:c r="AI9" s="26" t="n">
         <x:f>AVERAGE(Y9:AD9)</x:f>
         <x:v>66.66666666666667</x:v>
       </x:c>
-      <x:c r="AJ9" s="10" t="n">
+      <x:c r="AJ9" s="26" t="n">
         <x:f>SUMPRODUCT(AE9:AI9,Overview!$B$34:$F$34)</x:f>
         <x:v>71.39285714285714</x:v>
       </x:c>
-      <x:c r="AK9" s="10" t="n">
+      <x:c r="AK9" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ9-$AJ$25)/$AJ$26)</x:f>
         <x:v>77.47984409217784</x:v>
       </x:c>
-      <x:c r="AL9" s="10" t="n">
+      <x:c r="AL9" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK9-AJ9)</x:f>
         <x:v>6.086986949320703</x:v>
       </x:c>
@@ -2632,6 +2733,22 @@
       <x:c r="AP9" s="8" t="str">
         <x:v>d0c5b7842bae624f6bdf113976977c635367ecd9</x:v>
       </x:c>
+      <x:c r="AQ9" s="33" t="n">
+        <x:f>AR9+IF(AT9&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="AR9" s="33" t="n">
+        <x:f>INT(AK9)</x:f>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="AS9" s="35" t="n">
+        <x:f>AK9-AR9</x:f>
+        <x:v>0.4798440921778422</x:v>
+      </x:c>
+      <x:c r="AT9" s="33" t="n">
+        <x:f>RANK(AS9,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS9,AS9)-1</x:f>
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="2" t="str">
@@ -2724,35 +2841,35 @@
       <x:c r="AD10" s="18" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="AE10" s="9" t="n">
+      <x:c r="AE10" s="25" t="n">
         <x:f>AVERAGE(B10:F10)</x:f>
         <x:v>69</x:v>
       </x:c>
-      <x:c r="AF10" s="9" t="n">
+      <x:c r="AF10" s="25" t="n">
         <x:f>AVERAGE(G10:L10)</x:f>
         <x:v>69.16666666666667</x:v>
       </x:c>
-      <x:c r="AG10" s="9" t="n">
+      <x:c r="AG10" s="25" t="n">
         <x:f>AVERAGE(M10:Q10)</x:f>
         <x:v>68</x:v>
       </x:c>
-      <x:c r="AH10" s="9" t="n">
+      <x:c r="AH10" s="25" t="n">
         <x:f>AVERAGE(R10:X10)</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="AI10" s="9" t="n">
+      <x:c r="AI10" s="25" t="n">
         <x:f>AVERAGE(Y10:AD10)</x:f>
         <x:v>67.5</x:v>
       </x:c>
-      <x:c r="AJ10" s="9" t="n">
+      <x:c r="AJ10" s="25" t="n">
         <x:f>SUMPRODUCT(AE10:AI10,Overview!$B$34:$F$34)</x:f>
         <x:v>68.5952380952381</x:v>
       </x:c>
-      <x:c r="AK10" s="9" t="n">
+      <x:c r="AK10" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ10-$AJ$25)/$AJ$26)</x:f>
         <x:v>74.28480566427241</x:v>
       </x:c>
-      <x:c r="AL10" s="9" t="n">
+      <x:c r="AL10" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK10-AJ10)</x:f>
         <x:v>5.68956756903431</x:v>
       </x:c>
@@ -2767,6 +2884,22 @@
       <x:c r="AP10" s="2" t="str">
         <x:v>6c996dd073644346ccf058536400b96750bdf99a</x:v>
       </x:c>
+      <x:c r="AQ10" s="32" t="n">
+        <x:f>AR10+IF(AT10&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="AR10" s="32" t="n">
+        <x:f>INT(AK10)</x:f>
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="AS10" s="34" t="n">
+        <x:f>AK10-AR10</x:f>
+        <x:v>0.2848056642724117</x:v>
+      </x:c>
+      <x:c r="AT10" s="32" t="n">
+        <x:f>RANK(AS10,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS10,AS10)-1</x:f>
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="8" t="str">
@@ -2859,35 +2992,35 @@
       <x:c r="AD11" s="19" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="AE11" s="10" t="n">
+      <x:c r="AE11" s="26" t="n">
         <x:f>AVERAGE(B11:F11)</x:f>
         <x:v>59</x:v>
       </x:c>
-      <x:c r="AF11" s="10" t="n">
+      <x:c r="AF11" s="26" t="n">
         <x:f>AVERAGE(G11:L11)</x:f>
         <x:v>74.16666666666667</x:v>
       </x:c>
-      <x:c r="AG11" s="10" t="n">
+      <x:c r="AG11" s="26" t="n">
         <x:f>AVERAGE(M11:Q11)</x:f>
         <x:v>74</x:v>
       </x:c>
-      <x:c r="AH11" s="10" t="n">
+      <x:c r="AH11" s="26" t="n">
         <x:f>AVERAGE(R11:X11)</x:f>
         <x:v>70.71428571428571</x:v>
       </x:c>
-      <x:c r="AI11" s="10" t="n">
+      <x:c r="AI11" s="26" t="n">
         <x:f>AVERAGE(Y11:AD11)</x:f>
         <x:v>68.33333333333333</x:v>
       </x:c>
-      <x:c r="AJ11" s="10" t="n">
+      <x:c r="AJ11" s="26" t="n">
         <x:f>SUMPRODUCT(AE11:AI11,Overview!$B$34:$F$34)</x:f>
         <x:v>69.11309523809524</x:v>
       </x:c>
-      <x:c r="AK11" s="10" t="n">
+      <x:c r="AK11" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ11-$AJ$25)/$AJ$26)</x:f>
         <x:v>74.87622767114001</x:v>
       </x:c>
-      <x:c r="AL11" s="10" t="n">
+      <x:c r="AL11" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK11-AJ11)</x:f>
         <x:v>5.763132433044774</x:v>
       </x:c>
@@ -2902,6 +3035,22 @@
       <x:c r="AP11" s="8" t="str">
         <x:v>cc7b0426b6759e81ad0926a7357155e34abcc7f2</x:v>
       </x:c>
+      <x:c r="AQ11" s="33" t="n">
+        <x:f>AR11+IF(AT11&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="AR11" s="33" t="n">
+        <x:f>INT(AK11)</x:f>
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="AS11" s="35" t="n">
+        <x:f>AK11-AR11</x:f>
+        <x:v>0.8762276711400148</x:v>
+      </x:c>
+      <x:c r="AT11" s="33" t="n">
+        <x:f>RANK(AS11,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS11,AS11)-1</x:f>
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="2" t="str">
@@ -2994,35 +3143,35 @@
       <x:c r="AD12" s="18" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="AE12" s="9" t="n">
+      <x:c r="AE12" s="25" t="n">
         <x:f>AVERAGE(B12:F12)</x:f>
         <x:v>43</x:v>
       </x:c>
-      <x:c r="AF12" s="9" t="n">
+      <x:c r="AF12" s="25" t="n">
         <x:f>AVERAGE(G12:L12)</x:f>
         <x:v>45</x:v>
       </x:c>
-      <x:c r="AG12" s="9" t="n">
+      <x:c r="AG12" s="25" t="n">
         <x:f>AVERAGE(M12:Q12)</x:f>
         <x:v>49</x:v>
       </x:c>
-      <x:c r="AH12" s="9" t="n">
+      <x:c r="AH12" s="25" t="n">
         <x:f>AVERAGE(R12:X12)</x:f>
         <x:v>57.857142857142854</x:v>
       </x:c>
-      <x:c r="AI12" s="9" t="n">
+      <x:c r="AI12" s="25" t="n">
         <x:f>AVERAGE(Y12:AD12)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AJ12" s="9" t="n">
+      <x:c r="AJ12" s="25" t="n">
         <x:f>SUMPRODUCT(AE12:AI12,Overview!$B$34:$F$34)</x:f>
         <x:v>49.035714285714285</x:v>
       </x:c>
-      <x:c r="AK12" s="9" t="n">
+      <x:c r="AK12" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ12-$AJ$25)/$AJ$26)</x:f>
         <x:v>51.94672848534201</x:v>
       </x:c>
-      <x:c r="AL12" s="9" t="n">
+      <x:c r="AL12" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK12-AJ12)</x:f>
         <x:v>2.911014199627722</x:v>
       </x:c>
@@ -3037,6 +3186,22 @@
       <x:c r="AP12" s="2" t="str">
         <x:v>150cc055bff299f5d08dff97f1f1f631c1420416</x:v>
       </x:c>
+      <x:c r="AQ12" s="32" t="n">
+        <x:f>AR12+IF(AT12&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="AR12" s="32" t="n">
+        <x:f>INT(AK12)</x:f>
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="AS12" s="34" t="n">
+        <x:f>AK12-AR12</x:f>
+        <x:v>0.9467284853420068</x:v>
+      </x:c>
+      <x:c r="AT12" s="32" t="n">
+        <x:f>RANK(AS12,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS12,AS12)-1</x:f>
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="8" t="str">
@@ -3129,35 +3294,35 @@
       <x:c r="AD13" s="19" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="AE13" s="10" t="n">
+      <x:c r="AE13" s="26" t="n">
         <x:f>AVERAGE(B13:F13)</x:f>
         <x:v>44</x:v>
       </x:c>
-      <x:c r="AF13" s="10" t="n">
+      <x:c r="AF13" s="26" t="n">
         <x:f>AVERAGE(G13:L13)</x:f>
         <x:v>48.333333333333336</x:v>
       </x:c>
-      <x:c r="AG13" s="10" t="n">
+      <x:c r="AG13" s="26" t="n">
         <x:f>AVERAGE(M13:Q13)</x:f>
         <x:v>52</x:v>
       </x:c>
-      <x:c r="AH13" s="10" t="n">
+      <x:c r="AH13" s="26" t="n">
         <x:f>AVERAGE(R13:X13)</x:f>
         <x:v>60.714285714285715</x:v>
       </x:c>
-      <x:c r="AI13" s="10" t="n">
+      <x:c r="AI13" s="26" t="n">
         <x:f>AVERAGE(Y13:AD13)</x:f>
         <x:v>30</x:v>
       </x:c>
-      <x:c r="AJ13" s="10" t="n">
+      <x:c r="AJ13" s="26" t="n">
         <x:f>SUMPRODUCT(AE13:AI13,Overview!$B$34:$F$34)</x:f>
         <x:v>46.654761904761905</x:v>
       </x:c>
-      <x:c r="AK13" s="10" t="n">
+      <x:c r="AK13" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ13-$AJ$25)/$AJ$26)</x:f>
         <x:v>49.22754684457142</x:v>
       </x:c>
-      <x:c r="AL13" s="10" t="n">
+      <x:c r="AL13" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK13-AJ13)</x:f>
         <x:v>2.572784939809516</x:v>
       </x:c>
@@ -3172,6 +3337,22 @@
       <x:c r="AP13" s="8" t="str">
         <x:v>ed0986287bebdc2a51c00d9187aba269a380a677</x:v>
       </x:c>
+      <x:c r="AQ13" s="33" t="n">
+        <x:f>AR13+IF(AT13&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="AR13" s="33" t="n">
+        <x:f>INT(AK13)</x:f>
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="AS13" s="35" t="n">
+        <x:f>AK13-AR13</x:f>
+        <x:v>0.22754684457142105</x:v>
+      </x:c>
+      <x:c r="AT13" s="33" t="n">
+        <x:f>RANK(AS13,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS13,AS13)-1</x:f>
+        <x:v>15</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="2" t="str">
@@ -3264,35 +3445,35 @@
       <x:c r="AD14" s="18" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="AE14" s="9" t="n">
+      <x:c r="AE14" s="25" t="n">
         <x:f>AVERAGE(B14:F14)</x:f>
         <x:v>43</x:v>
       </x:c>
-      <x:c r="AF14" s="9" t="n">
+      <x:c r="AF14" s="25" t="n">
         <x:f>AVERAGE(G14:L14)</x:f>
         <x:v>54.166666666666664</x:v>
       </x:c>
-      <x:c r="AG14" s="9" t="n">
+      <x:c r="AG14" s="25" t="n">
         <x:f>AVERAGE(M14:Q14)</x:f>
         <x:v>53</x:v>
       </x:c>
-      <x:c r="AH14" s="9" t="n">
+      <x:c r="AH14" s="25" t="n">
         <x:f>AVERAGE(R14:X14)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AI14" s="9" t="n">
+      <x:c r="AI14" s="25" t="n">
         <x:f>AVERAGE(Y14:AD14)</x:f>
         <x:v>59.166666666666664</x:v>
       </x:c>
-      <x:c r="AJ14" s="9" t="n">
+      <x:c r="AJ14" s="25" t="n">
         <x:f>SUMPRODUCT(AE14:AI14,Overview!$B$34:$F$34)</x:f>
         <x:v>52.416666666666664</x:v>
       </x:c>
-      <x:c r="AK14" s="9" t="n">
+      <x:c r="AK14" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ14-$AJ$25)/$AJ$26)</x:f>
         <x:v>55.807966415236244</x:v>
       </x:c>
-      <x:c r="AL14" s="9" t="n">
+      <x:c r="AL14" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK14-AJ14)</x:f>
         <x:v>3.3912997485695797</x:v>
       </x:c>
@@ -3307,6 +3488,22 @@
       <x:c r="AP14" s="2" t="str">
         <x:v>24155530889c12af50c61eb5900c811090e440cd</x:v>
       </x:c>
+      <x:c r="AQ14" s="32" t="n">
+        <x:f>AR14+IF(AT14&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="AR14" s="32" t="n">
+        <x:f>INT(AK14)</x:f>
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="AS14" s="34" t="n">
+        <x:f>AK14-AR14</x:f>
+        <x:v>0.807966415236244</x:v>
+      </x:c>
+      <x:c r="AT14" s="32" t="n">
+        <x:f>RANK(AS14,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS14,AS14)-1</x:f>
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="8" t="str">
@@ -3399,35 +3596,35 @@
       <x:c r="AD15" s="19" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="AE15" s="10" t="n">
+      <x:c r="AE15" s="26" t="n">
         <x:f>AVERAGE(B15:F15)</x:f>
         <x:v>72</x:v>
       </x:c>
-      <x:c r="AF15" s="10" t="n">
+      <x:c r="AF15" s="26" t="n">
         <x:f>AVERAGE(G15:L15)</x:f>
         <x:v>82.5</x:v>
       </x:c>
-      <x:c r="AG15" s="10" t="n">
+      <x:c r="AG15" s="26" t="n">
         <x:f>AVERAGE(M15:Q15)</x:f>
         <x:v>74</x:v>
       </x:c>
-      <x:c r="AH15" s="10" t="n">
+      <x:c r="AH15" s="26" t="n">
         <x:f>AVERAGE(R15:X15)</x:f>
         <x:v>76.42857142857143</x:v>
       </x:c>
-      <x:c r="AI15" s="10" t="n">
+      <x:c r="AI15" s="26" t="n">
         <x:f>AVERAGE(Y15:AD15)</x:f>
         <x:v>71.66666666666667</x:v>
       </x:c>
-      <x:c r="AJ15" s="10" t="n">
+      <x:c r="AJ15" s="26" t="n">
         <x:f>SUMPRODUCT(AE15:AI15,Overview!$B$34:$F$34)</x:f>
         <x:v>75.51785714285714</x:v>
       </x:c>
-      <x:c r="AK15" s="10" t="n">
+      <x:c r="AK15" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ15-$AJ$25)/$AJ$26)</x:f>
         <x:v>82.19082628481289</x:v>
       </x:c>
-      <x:c r="AL15" s="10" t="n">
+      <x:c r="AL15" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK15-AJ15)</x:f>
         <x:v>6.672969141955747</x:v>
       </x:c>
@@ -3442,6 +3639,22 @@
       <x:c r="AP15" s="8" t="str">
         <x:v>b545607a9ce1c184ce7e2d09a34940464de27d26</x:v>
       </x:c>
+      <x:c r="AQ15" s="33" t="n">
+        <x:f>AR15+IF(AT15&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="AR15" s="33" t="n">
+        <x:f>INT(AK15)</x:f>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="AS15" s="35" t="n">
+        <x:f>AK15-AR15</x:f>
+        <x:v>0.19082628481288566</x:v>
+      </x:c>
+      <x:c r="AT15" s="33" t="n">
+        <x:f>RANK(AS15,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS15,AS15)-1</x:f>
+        <x:v>16</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="2" t="str">
@@ -3534,35 +3747,35 @@
       <x:c r="AD16" s="18" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="AE16" s="9" t="n">
+      <x:c r="AE16" s="25" t="n">
         <x:f>AVERAGE(B16:F16)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AF16" s="9" t="n">
+      <x:c r="AF16" s="25" t="n">
         <x:f>AVERAGE(G16:L16)</x:f>
         <x:v>75</x:v>
       </x:c>
-      <x:c r="AG16" s="9" t="n">
+      <x:c r="AG16" s="25" t="n">
         <x:f>AVERAGE(M16:Q16)</x:f>
         <x:v>73</x:v>
       </x:c>
-      <x:c r="AH16" s="9" t="n">
+      <x:c r="AH16" s="25" t="n">
         <x:f>AVERAGE(R16:X16)</x:f>
         <x:v>76.42857142857143</x:v>
       </x:c>
-      <x:c r="AI16" s="9" t="n">
+      <x:c r="AI16" s="25" t="n">
         <x:f>AVERAGE(Y16:AD16)</x:f>
         <x:v>73.33333333333333</x:v>
       </x:c>
-      <x:c r="AJ16" s="9" t="n">
+      <x:c r="AJ16" s="25" t="n">
         <x:f>SUMPRODUCT(AE16:AI16,Overview!$B$34:$F$34)</x:f>
         <x:v>70.64285714285714</x:v>
       </x:c>
-      <x:c r="AK16" s="9" t="n">
+      <x:c r="AK16" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ16-$AJ$25)/$AJ$26)</x:f>
         <x:v>76.6233018753351</x:v>
       </x:c>
-      <x:c r="AL16" s="9" t="n">
+      <x:c r="AL16" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK16-AJ16)</x:f>
         <x:v>5.980444732477963</x:v>
       </x:c>
@@ -3577,6 +3790,22 @@
       <x:c r="AP16" s="2" t="str">
         <x:v>51304fe042179d309e97bb1999af5e9201f8dae8</x:v>
       </x:c>
+      <x:c r="AQ16" s="32" t="n">
+        <x:f>AR16+IF(AT16&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="AR16" s="32" t="n">
+        <x:f>INT(AK16)</x:f>
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="AS16" s="34" t="n">
+        <x:f>AK16-AR16</x:f>
+        <x:v>0.6233018753351018</x:v>
+      </x:c>
+      <x:c r="AT16" s="32" t="n">
+        <x:f>RANK(AS16,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS16,AS16)-1</x:f>
+        <x:v>8</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="8" t="str">
@@ -3669,35 +3898,35 @@
       <x:c r="AD17" s="19" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="AE17" s="10" t="n">
+      <x:c r="AE17" s="26" t="n">
         <x:f>AVERAGE(B17:F17)</x:f>
         <x:v>52</x:v>
       </x:c>
-      <x:c r="AF17" s="10" t="n">
+      <x:c r="AF17" s="26" t="n">
         <x:f>AVERAGE(G17:L17)</x:f>
         <x:v>51.666666666666664</x:v>
       </x:c>
-      <x:c r="AG17" s="10" t="n">
+      <x:c r="AG17" s="26" t="n">
         <x:f>AVERAGE(M17:Q17)</x:f>
         <x:v>63</x:v>
       </x:c>
-      <x:c r="AH17" s="10" t="n">
+      <x:c r="AH17" s="26" t="n">
         <x:f>AVERAGE(R17:X17)</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="AI17" s="10" t="n">
+      <x:c r="AI17" s="26" t="n">
         <x:f>AVERAGE(Y17:AD17)</x:f>
         <x:v>60.833333333333336</x:v>
       </x:c>
-      <x:c r="AJ17" s="10" t="n">
+      <x:c r="AJ17" s="26" t="n">
         <x:f>SUMPRODUCT(AE17:AI17,Overview!$B$34:$F$34)</x:f>
         <x:v>57.720238095238095</x:v>
       </x:c>
-      <x:c r="AK17" s="10" t="n">
+      <x:c r="AK17" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ17-$AJ$25)/$AJ$26)</x:f>
         <x:v>61.864943520052734</x:v>
       </x:c>
-      <x:c r="AL17" s="10" t="n">
+      <x:c r="AL17" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK17-AJ17)</x:f>
         <x:v>4.144705424814639</x:v>
       </x:c>
@@ -3712,6 +3941,22 @@
       <x:c r="AP17" s="8" t="str">
         <x:v>224f4343365132310337c919cbc4e32582f70cc9</x:v>
       </x:c>
+      <x:c r="AQ17" s="33" t="n">
+        <x:f>AR17+IF(AT17&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="AR17" s="33" t="n">
+        <x:f>INT(AK17)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="AS17" s="35" t="n">
+        <x:f>AK17-AR17</x:f>
+        <x:v>0.8649435200527336</x:v>
+      </x:c>
+      <x:c r="AT17" s="33" t="n">
+        <x:f>RANK(AS17,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS17,AS17)-1</x:f>
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="2" t="str">
@@ -3804,35 +4049,35 @@
       <x:c r="AD18" s="18" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="AE18" s="9" t="n">
+      <x:c r="AE18" s="25" t="n">
         <x:f>AVERAGE(B18:F18)</x:f>
         <x:v>37</x:v>
       </x:c>
-      <x:c r="AF18" s="9" t="n">
+      <x:c r="AF18" s="25" t="n">
         <x:f>AVERAGE(G18:L18)</x:f>
         <x:v>55.833333333333336</x:v>
       </x:c>
-      <x:c r="AG18" s="9" t="n">
+      <x:c r="AG18" s="25" t="n">
         <x:f>AVERAGE(M18:Q18)</x:f>
         <x:v>57</x:v>
       </x:c>
-      <x:c r="AH18" s="9" t="n">
+      <x:c r="AH18" s="25" t="n">
         <x:f>AVERAGE(R18:X18)</x:f>
         <x:v>57.857142857142854</x:v>
       </x:c>
-      <x:c r="AI18" s="9" t="n">
+      <x:c r="AI18" s="25" t="n">
         <x:f>AVERAGE(Y18:AD18)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AJ18" s="9" t="n">
+      <x:c r="AJ18" s="25" t="n">
         <x:f>SUMPRODUCT(AE18:AI18,Overview!$B$34:$F$34)</x:f>
         <x:v>52.24404761904762</x:v>
       </x:c>
-      <x:c r="AK18" s="9" t="n">
+      <x:c r="AK18" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ18-$AJ$25)/$AJ$26)</x:f>
         <x:v>55.61082574628038</x:v>
       </x:c>
-      <x:c r="AL18" s="9" t="n">
+      <x:c r="AL18" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK18-AJ18)</x:f>
         <x:v>3.366778127232763</x:v>
       </x:c>
@@ -3847,6 +4092,22 @@
       <x:c r="AP18" s="2" t="str">
         <x:v>37b040a376a923dd4ad28fa07532e223d8f87385</x:v>
       </x:c>
+      <x:c r="AQ18" s="32" t="n">
+        <x:f>AR18+IF(AT18&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="AR18" s="32" t="n">
+        <x:f>INT(AK18)</x:f>
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="AS18" s="34" t="n">
+        <x:f>AK18-AR18</x:f>
+        <x:v>0.6108257462803834</x:v>
+      </x:c>
+      <x:c r="AT18" s="32" t="n">
+        <x:f>RANK(AS18,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS18,AS18)-1</x:f>
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="8" t="str">
@@ -3939,35 +4200,35 @@
       <x:c r="AD19" s="19" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="AE19" s="10" t="n">
+      <x:c r="AE19" s="26" t="n">
         <x:f>AVERAGE(B19:F19)</x:f>
         <x:v>39</x:v>
       </x:c>
-      <x:c r="AF19" s="10" t="n">
+      <x:c r="AF19" s="26" t="n">
         <x:f>AVERAGE(G19:L19)</x:f>
         <x:v>62.5</x:v>
       </x:c>
-      <x:c r="AG19" s="10" t="n">
+      <x:c r="AG19" s="26" t="n">
         <x:f>AVERAGE(M19:Q19)</x:f>
         <x:v>63</x:v>
       </x:c>
-      <x:c r="AH19" s="10" t="n">
+      <x:c r="AH19" s="26" t="n">
         <x:f>AVERAGE(R19:X19)</x:f>
         <x:v>69.28571428571429</x:v>
       </x:c>
-      <x:c r="AI19" s="10" t="n">
+      <x:c r="AI19" s="26" t="n">
         <x:f>AVERAGE(Y19:AD19)</x:f>
         <x:v>62.5</x:v>
       </x:c>
-      <x:c r="AJ19" s="10" t="n">
+      <x:c r="AJ19" s="26" t="n">
         <x:f>SUMPRODUCT(AE19:AI19,Overview!$B$34:$F$34)</x:f>
         <x:v>57.42857142857143</x:v>
       </x:c>
-      <x:c r="AK19" s="10" t="n">
+      <x:c r="AK19" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ19-$AJ$25)/$AJ$26)</x:f>
         <x:v>61.53184376905834</x:v>
       </x:c>
-      <x:c r="AL19" s="10" t="n">
+      <x:c r="AL19" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK19-AJ19)</x:f>
         <x:v>4.10327234048691</x:v>
       </x:c>
@@ -3982,6 +4243,22 @@
       <x:c r="AP19" s="8" t="str">
         <x:v>9fc7a1490c966cb547f30cd92e5bd5eafebfe014</x:v>
       </x:c>
+      <x:c r="AQ19" s="33" t="n">
+        <x:f>AR19+IF(AT19&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="AR19" s="33" t="n">
+        <x:f>INT(AK19)</x:f>
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="AS19" s="35" t="n">
+        <x:f>AK19-AR19</x:f>
+        <x:v>0.5318437690583409</x:v>
+      </x:c>
+      <x:c r="AT19" s="33" t="n">
+        <x:f>RANK(AS19,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS19,AS19)-1</x:f>
+        <x:v>11</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="2" t="str">
@@ -4074,35 +4351,35 @@
       <x:c r="AD20" s="18" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="AE20" s="9" t="n">
+      <x:c r="AE20" s="25" t="n">
         <x:f>AVERAGE(B20:F20)</x:f>
         <x:v>39</x:v>
       </x:c>
-      <x:c r="AF20" s="9" t="n">
+      <x:c r="AF20" s="25" t="n">
         <x:f>AVERAGE(G20:L20)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AG20" s="9" t="n">
+      <x:c r="AG20" s="25" t="n">
         <x:f>AVERAGE(M20:Q20)</x:f>
         <x:v>60</x:v>
       </x:c>
-      <x:c r="AH20" s="9" t="n">
+      <x:c r="AH20" s="25" t="n">
         <x:f>AVERAGE(R20:X20)</x:f>
         <x:v>57.857142857142854</x:v>
       </x:c>
-      <x:c r="AI20" s="9" t="n">
+      <x:c r="AI20" s="25" t="n">
         <x:f>AVERAGE(Y20:AD20)</x:f>
         <x:v>61.666666666666664</x:v>
       </x:c>
-      <x:c r="AJ20" s="9" t="n">
+      <x:c r="AJ20" s="25" t="n">
         <x:f>SUMPRODUCT(AE20:AI20,Overview!$B$34:$F$34)</x:f>
         <x:v>54.785714285714285</x:v>
       </x:c>
-      <x:c r="AK20" s="9" t="n">
+      <x:c r="AK20" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ20-$AJ$25)/$AJ$26)</x:f>
         <x:v>58.51355214780298</x:v>
       </x:c>
-      <x:c r="AL20" s="9" t="n">
+      <x:c r="AL20" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK20-AJ20)</x:f>
         <x:v>3.7278378620886983</x:v>
       </x:c>
@@ -4117,6 +4394,22 @@
       <x:c r="AP20" s="2" t="str">
         <x:v>8f73d864af17d2aec636cce960724975747b53e2</x:v>
       </x:c>
+      <x:c r="AQ20" s="32" t="n">
+        <x:f>AR20+IF(AT20&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="AR20" s="32" t="n">
+        <x:f>INT(AK20)</x:f>
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="AS20" s="34" t="n">
+        <x:f>AK20-AR20</x:f>
+        <x:v>0.513552147802983</x:v>
+      </x:c>
+      <x:c r="AT20" s="32" t="n">
+        <x:f>RANK(AS20,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS20,AS20)-1</x:f>
+        <x:v>12</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="8" t="str">
@@ -4209,35 +4502,35 @@
       <x:c r="AD21" s="19" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="AE21" s="10" t="n">
+      <x:c r="AE21" s="26" t="n">
         <x:f>AVERAGE(B21:F21)</x:f>
         <x:v>41</x:v>
       </x:c>
-      <x:c r="AF21" s="10" t="n">
+      <x:c r="AF21" s="26" t="n">
         <x:f>AVERAGE(G21:L21)</x:f>
         <x:v>70</x:v>
       </x:c>
-      <x:c r="AG21" s="10" t="n">
+      <x:c r="AG21" s="26" t="n">
         <x:f>AVERAGE(M21:Q21)</x:f>
         <x:v>67</x:v>
       </x:c>
-      <x:c r="AH21" s="10" t="n">
+      <x:c r="AH21" s="26" t="n">
         <x:f>AVERAGE(R21:X21)</x:f>
         <x:v>61.42857142857143</x:v>
       </x:c>
-      <x:c r="AI21" s="10" t="n">
+      <x:c r="AI21" s="26" t="n">
         <x:f>AVERAGE(Y21:AD21)</x:f>
         <x:v>69.16666666666667</x:v>
       </x:c>
-      <x:c r="AJ21" s="10" t="n">
+      <x:c r="AJ21" s="26" t="n">
         <x:f>SUMPRODUCT(AE21:AI21,Overview!$B$34:$F$34)</x:f>
         <x:v>61.017857142857146</x:v>
       </x:c>
-      <x:c r="AK21" s="10" t="n">
+      <x:c r="AK21" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ21-$AJ$25)/$AJ$26)</x:f>
         <x:v>65.63101009252</x:v>
       </x:c>
-      <x:c r="AL21" s="10" t="n">
+      <x:c r="AL21" s="26" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK21-AJ21)</x:f>
         <x:v>4.6131529496628545</x:v>
       </x:c>
@@ -4252,6 +4545,22 @@
       <x:c r="AP21" s="8" t="str">
         <x:v>05dcec9b74e99867ad6cf4cd9c14f858fecc8178</x:v>
       </x:c>
+      <x:c r="AQ21" s="33" t="n">
+        <x:f>AR21+IF(AT21&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="AR21" s="33" t="n">
+        <x:f>INT(AK21)</x:f>
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="AS21" s="35" t="n">
+        <x:f>AK21-AR21</x:f>
+        <x:v>0.6310100925200004</x:v>
+      </x:c>
+      <x:c r="AT21" s="33" t="n">
+        <x:f>RANK(AS21,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS21,AS21)-1</x:f>
+        <x:v>7</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="2" t="str">
@@ -4344,35 +4653,35 @@
       <x:c r="AD22" s="18" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="AE22" s="9" t="n">
+      <x:c r="AE22" s="25" t="n">
         <x:f>AVERAGE(B22:F22)</x:f>
         <x:v>47</x:v>
       </x:c>
-      <x:c r="AF22" s="9" t="n">
+      <x:c r="AF22" s="25" t="n">
         <x:f>AVERAGE(G22:L22)</x:f>
         <x:v>52.5</x:v>
       </x:c>
-      <x:c r="AG22" s="9" t="n">
+      <x:c r="AG22" s="25" t="n">
         <x:f>AVERAGE(M22:Q22)</x:f>
         <x:v>58</x:v>
       </x:c>
-      <x:c r="AH22" s="9" t="n">
+      <x:c r="AH22" s="25" t="n">
         <x:f>AVERAGE(R22:X22)</x:f>
         <x:v>61.42857142857143</x:v>
       </x:c>
-      <x:c r="AI22" s="9" t="n">
+      <x:c r="AI22" s="25" t="n">
         <x:f>AVERAGE(Y22:AD22)</x:f>
         <x:v>52.5</x:v>
       </x:c>
-      <x:c r="AJ22" s="9" t="n">
+      <x:c r="AJ22" s="25" t="n">
         <x:f>SUMPRODUCT(AE22:AI22,Overview!$B$34:$F$34)</x:f>
         <x:v>53.392857142857146</x:v>
       </x:c>
-      <x:c r="AK22" s="9" t="n">
+      <x:c r="AK22" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",Overview!$B$37+Overview!$B$38*(AJ22-$AJ$25)/$AJ$26)</x:f>
         <x:v>56.92283088795219</x:v>
       </x:c>
-      <x:c r="AL22" s="9" t="n">
+      <x:c r="AL22" s="25" t="n">
         <x:f>IF($AJ$26=0,"Undefined",AK22-AJ22)</x:f>
         <x:v>3.5299737450950417</x:v>
       </x:c>
@@ -4386,6 +4695,22 @@
       </x:c>
       <x:c r="AP22" s="2" t="str">
         <x:v>699e46315f5534e53299ef301971c364b9e4041b</x:v>
+      </x:c>
+      <x:c r="AQ22" s="32" t="n">
+        <x:f>AR22+IF(AT22&lt;=Overview!$B$37*COUNT($AJ$6:$AJ$22)-SUM($AR$6:$AR$22),1,0)</x:f>
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="AR22" s="32" t="n">
+        <x:f>INT(AK22)</x:f>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="AS22" s="34" t="n">
+        <x:f>AK22-AR22</x:f>
+        <x:v>0.9228308879521876</x:v>
+      </x:c>
+      <x:c r="AT22" s="32" t="n">
+        <x:f>RANK(AS22,$AS$6:$AS$22,0)+COUNTIF($AS$6:AS22,AS22)-1</x:f>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
@@ -4431,6 +4756,10 @@
       <x:c r="AN23" s="2"/>
       <x:c r="AO23" s="2"/>
       <x:c r="AP23" s="2"/>
+      <x:c r="AQ23" s="1"/>
+      <x:c r="AR23" s="1"/>
+      <x:c r="AS23" s="1"/>
+      <x:c r="AT23" s="1"/>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="2"/>
@@ -4475,6 +4804,10 @@
       <x:c r="AN24" s="2"/>
       <x:c r="AO24" s="2"/>
       <x:c r="AP24" s="2"/>
+      <x:c r="AQ24" s="1"/>
+      <x:c r="AR24" s="1"/>
+      <x:c r="AS24" s="1"/>
+      <x:c r="AT24" s="1"/>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="2" t="str">
@@ -4632,6 +4965,13 @@
       <x:c r="AN25" s="2"/>
       <x:c r="AO25" s="2"/>
       <x:c r="AP25" s="2"/>
+      <x:c r="AQ25" s="36" t="n">
+        <x:f>AVERAGE(AQ6:AQ22)</x:f>
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="AR25" s="1"/>
+      <x:c r="AS25" s="1"/>
+      <x:c r="AT25" s="1"/>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="2" t="str">
@@ -4789,6 +5129,13 @@
       <x:c r="AN26" s="2"/>
       <x:c r="AO26" s="2"/>
       <x:c r="AP26" s="2"/>
+      <x:c r="AQ26" s="36" t="n">
+        <x:f>STDEV.P(AQ6:AQ22)</x:f>
+        <x:v>9.952829925674997</x:v>
+      </x:c>
+      <x:c r="AR26" s="1"/>
+      <x:c r="AS26" s="1"/>
+      <x:c r="AT26" s="1"/>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="2" t="str">
@@ -4946,6 +5293,13 @@
       <x:c r="AN27" s="2"/>
       <x:c r="AO27" s="2"/>
       <x:c r="AP27" s="2"/>
+      <x:c r="AQ27" s="36" t="n">
+        <x:f>MIN(AQ6:AQ22)</x:f>
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="AR27" s="1"/>
+      <x:c r="AS27" s="1"/>
+      <x:c r="AT27" s="1"/>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="2" t="str">
@@ -5103,6 +5457,13 @@
       <x:c r="AN28" s="2"/>
       <x:c r="AO28" s="2"/>
       <x:c r="AP28" s="2"/>
+      <x:c r="AQ28" s="36" t="n">
+        <x:f>MAX(AQ6:AQ22)</x:f>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="AR28" s="1"/>
+      <x:c r="AS28" s="1"/>
+      <x:c r="AT28" s="1"/>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="2"/>
@@ -6374,10 +6735,10 @@
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
       <x:c r="A42" s="2" t="str">
-        <x:v>Comparison</x:v>
+        <x:v>Standardised</x:v>
       </x:c>
       <x:c r="B42" s="2" t="str">
-        <x:v>Separate standardised overall</x:v>
+        <x:v>Overall before final integer rounding</x:v>
       </x:c>
       <x:c r="C42" s="2" t="n">
         <x:f>COUNT('Subcriterion marks'!AK6:AK22)</x:f>
@@ -6400,6 +6761,35 @@
         <x:v>82.19082628481289</x:v>
       </x:c>
       <x:c r="H42" s="20"/>
+    </x:row>
+    <x:row r="43" ht="25" customHeight="1">
+      <x:c r="A43" s="1" t="str">
+        <x:v>Moderated</x:v>
+      </x:c>
+      <x:c r="B43" s="1" t="str">
+        <x:v>Mean-preserving whole-number overall</x:v>
+      </x:c>
+      <x:c r="C43" s="1" t="n">
+        <x:f>COUNT('Subcriterion marks'!AQ6:AQ22)</x:f>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D43" s="36" t="n">
+        <x:f>AVERAGE('Subcriterion marks'!AQ6:AQ22)</x:f>
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="E43" s="36" t="n">
+        <x:f>STDEV.P('Subcriterion marks'!AQ6:AQ22)</x:f>
+        <x:v>9.952829925674997</x:v>
+      </x:c>
+      <x:c r="F43" s="36" t="n">
+        <x:f>MIN('Subcriterion marks'!AQ6:AQ22)</x:f>
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="G43" s="36" t="n">
+        <x:f>MAX('Subcriterion marks'!AQ6:AQ22)</x:f>
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="H43" s="1"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>